<commit_message>
QA tracker: statuses after the 2026-10-13 release, plus new rows for games, the 1.0.0+8 features, the production stalls and the open decisions
28 App and 14 Panel rows moved from Fixed (in code) to Released (git shows their commits are in play-8 / panel main). New App rows 31-52 and Panel rows 18-23. 75 rows in total; Summary updates itself.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SABALIVE-QA-Tracker.xlsx
+++ b/SABALIVE-QA-Tracker.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Lists" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'App'!$A$1:$R$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Panel'!$A$1:$S$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'App'!$A$1:$R$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Panel'!$A$1:$S$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1098,7 +1098,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R31"/>
+  <dimension ref="A1:R53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1266,13 +1266,13 @@
       <c r="L2" s="11" t="inlineStr"/>
       <c r="M2" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="N2" s="11" t="inlineStr"/>
       <c r="O2" s="11" t="inlineStr">
         <is>
-          <t>Committed (Oct 2026 batch)</t>
+          <t>Committed (Oct 2026 batch) | Released: Play 1.0.0+8 (published to everyone 2026-10-13; commit is in tag play-8)</t>
         </is>
       </c>
       <c r="P2" s="11" t="inlineStr">
@@ -1283,7 +1283,7 @@
       <c r="Q2" s="11" t="inlineStr"/>
       <c r="R2" s="11" t="inlineStr">
         <is>
-          <t>Needs a Play release and re-submission to clear the policy issue.</t>
+          <t>Needs a Play release and re-submission to clear the policy issue. | Status set to Released on 2026-10-14 from git: this commit is in the source of Play 1.0.0+8. Not yet verified by a person.</t>
         </is>
       </c>
     </row>
@@ -1340,13 +1340,13 @@
       <c r="L3" s="11" t="inlineStr"/>
       <c r="M3" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="N3" s="11" t="inlineStr"/>
       <c r="O3" s="11" t="inlineStr">
         <is>
-          <t>ffb3369</t>
+          <t>ffb3369 | Released: Play 1.0.0+8 (published to everyone 2026-10-13; commit is in tag play-8)</t>
         </is>
       </c>
       <c r="P3" s="11" t="inlineStr">
@@ -1357,7 +1357,7 @@
       <c r="Q3" s="11" t="inlineStr"/>
       <c r="R3" s="11" t="inlineStr">
         <is>
-          <t>Test: test/keyboard_focus_test.dart.</t>
+          <t>Test: test/keyboard_focus_test.dart. | Status set to Released on 2026-10-14 from git: this commit is in the source of Play 1.0.0+8. Not yet verified by a person. | The commit is also in tag play-live (the 1.0.0+7 build).</t>
         </is>
       </c>
     </row>
@@ -1484,13 +1484,13 @@
       <c r="L5" s="11" t="inlineStr"/>
       <c r="M5" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="N5" s="11" t="inlineStr"/>
       <c r="O5" s="11" t="inlineStr">
         <is>
-          <t>5850a64 (DB) + ee1aed0 (app)</t>
+          <t>5850a64 (DB) + ee1aed0 (app) | Released: Play 1.0.0+8 (published to everyone 2026-10-13; commit is in tag play-8)</t>
         </is>
       </c>
       <c r="P5" s="11" t="inlineStr">
@@ -1501,7 +1501,7 @@
       <c r="Q5" s="11" t="inlineStr"/>
       <c r="R5" s="11" t="inlineStr">
         <is>
-          <t>Database part is live. App part ships in 1.0.0+8.</t>
+          <t>Database part is live. App part ships in 1.0.0+8. | Status set to Released on 2026-10-14 from git: this commit is in the source of Play 1.0.0+8. Not yet verified by a person.</t>
         </is>
       </c>
     </row>
@@ -1562,13 +1562,13 @@
       <c r="L6" s="11" t="inlineStr"/>
       <c r="M6" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="N6" s="11" t="inlineStr"/>
       <c r="O6" s="11" t="inlineStr">
         <is>
-          <t>5850a64 (DB) + ee1aed0 (app)</t>
+          <t>5850a64 (DB) + ee1aed0 (app) | Released: Play 1.0.0+8 (published to everyone 2026-10-13; commit is in tag play-8)</t>
         </is>
       </c>
       <c r="P6" s="11" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="R6" s="11" t="inlineStr">
         <is>
-          <t>DB part is live for existing builds (users must re-sit or rejoin). Waves UI ships in +8.</t>
+          <t>DB part is live for existing builds (users must re-sit or rejoin). Waves UI ships in +8. | Status set to Released on 2026-10-14 from git: this commit is in the source of Play 1.0.0+8. Not yet verified by a person.</t>
         </is>
       </c>
     </row>
@@ -1648,13 +1648,13 @@
       </c>
       <c r="M7" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="N7" s="11" t="inlineStr"/>
       <c r="O7" s="11" t="inlineStr">
         <is>
-          <t>ee1aed0</t>
+          <t>ee1aed0 | Released: Play 1.0.0+8 (published to everyone 2026-10-13; commit is in tag play-8)</t>
         </is>
       </c>
       <c r="P7" s="11" t="inlineStr">
@@ -1665,7 +1665,7 @@
       <c r="Q7" s="11" t="inlineStr"/>
       <c r="R7" s="11" t="inlineStr">
         <is>
-          <t>Shape is generated (Agora only reports loudness). Runs only while someone is heard.</t>
+          <t>Shape is generated (Agora only reports loudness). Runs only while someone is heard. | Status set to Released on 2026-10-14 from git: this commit is in the source of Play 1.0.0+8. Not yet verified by a person.</t>
         </is>
       </c>
     </row>
@@ -1726,13 +1726,13 @@
       <c r="L8" s="11" t="inlineStr"/>
       <c r="M8" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="N8" s="11" t="inlineStr"/>
       <c r="O8" s="11" t="inlineStr">
         <is>
-          <t>ee1aed0</t>
+          <t>ee1aed0 | Released: Play 1.0.0+8 (published to everyone 2026-10-13; commit is in tag play-8)</t>
         </is>
       </c>
       <c r="P8" s="11" t="inlineStr">
@@ -1743,7 +1743,7 @@
       <c r="Q8" s="11" t="inlineStr"/>
       <c r="R8" s="11" t="inlineStr">
         <is>
-          <t>Unit-tested only. Verify on a real Android 16 phone with gesture AND button navigation.</t>
+          <t>Unit-tested only. Verify on a real Android 16 phone with gesture AND button navigation. | Status set to Released on 2026-10-14 from git: this commit is in the source of Play 1.0.0+8. Not yet verified by a person.</t>
         </is>
       </c>
     </row>
@@ -1804,13 +1804,13 @@
       <c r="L9" s="11" t="inlineStr"/>
       <c r="M9" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="N9" s="11" t="inlineStr"/>
       <c r="O9" s="11" t="inlineStr">
         <is>
-          <t>ee1aed0</t>
+          <t>ee1aed0 | Released: Play 1.0.0+8 (published to everyone 2026-10-13; commit is in tag play-8)</t>
         </is>
       </c>
       <c r="P9" s="11" t="inlineStr">
@@ -1821,7 +1821,7 @@
       <c r="Q9" s="11" t="inlineStr"/>
       <c r="R9" s="11" t="inlineStr">
         <is>
-          <t>Not measured on a device. Next ideas: thermal-adaptive quality; lower video resolution (see the Agora cost item).</t>
+          <t>Not measured on a device. Next ideas: thermal-adaptive quality; lower video resolution (see the Agora cost item). | Status set to Released on 2026-10-14 from git: this commit is in the source of Play 1.0.0+8. Not yet verified by a person.</t>
         </is>
       </c>
     </row>
@@ -1960,13 +1960,13 @@
       <c r="L11" s="11" t="inlineStr"/>
       <c r="M11" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="N11" s="11" t="inlineStr"/>
       <c r="O11" s="11" t="inlineStr">
         <is>
-          <t>5850a64 (DB) + ee1aed0</t>
+          <t>5850a64 (DB) + ee1aed0 | Released: Play 1.0.0+8 (published to everyone 2026-10-13; commit is in tag play-8)</t>
         </is>
       </c>
       <c r="P11" s="11" t="inlineStr">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="R11" s="11" t="inlineStr">
         <is>
-          <t>Migration 20261004200000 is live.</t>
+          <t>Migration 20261004200000 is live. | Status set to Released on 2026-10-14 from git: this commit is in the source of Play 1.0.0+8. Not yet verified by a person.</t>
         </is>
       </c>
     </row>
@@ -2038,13 +2038,13 @@
       <c r="L12" s="11" t="inlineStr"/>
       <c r="M12" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="N12" s="11" t="inlineStr"/>
       <c r="O12" s="11" t="inlineStr">
         <is>
-          <t>5850a64</t>
+          <t>5850a64 | Released: Play 1.0.0+8 (published to everyone 2026-10-13; commit is in tag play-8)</t>
         </is>
       </c>
       <c r="P12" s="11" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="R12" s="11" t="inlineStr">
         <is>
-          <t>Kept closed on purpose when the rollback was discussed.</t>
+          <t>Kept closed on purpose when the rollback was discussed. | Status set to Released on 2026-10-14 from git: this commit is in the source of Play 1.0.0+8. Not yet verified by a person.</t>
         </is>
       </c>
     </row>
@@ -2124,13 +2124,13 @@
       </c>
       <c r="M13" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="N13" s="11" t="inlineStr"/>
       <c r="O13" s="11" t="inlineStr">
         <is>
-          <t>e5aa4f6</t>
+          <t>e5aa4f6 | Released: Play 1.0.0+8 (published to everyone 2026-10-13; commit is in tag play-8)</t>
         </is>
       </c>
       <c r="P13" s="11" t="inlineStr">
@@ -2141,7 +2141,7 @@
       <c r="Q13" s="11" t="inlineStr"/>
       <c r="R13" s="11" t="inlineStr">
         <is>
-          <t>Real cause on that phone unknown (Play Services?). Email, phone and username login are unaffected. Ask the reporter for model + Android version.</t>
+          <t>Real cause on that phone unknown (Play Services?). Email, phone and username login are unaffected. Ask the reporter for model + Android version. | Status set to Released on 2026-10-14 from git: this commit is in the source of Play 1.0.0+8. Not yet verified by a person.</t>
         </is>
       </c>
     </row>
@@ -2202,13 +2202,13 @@
       </c>
       <c r="M14" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="N14" s="11" t="inlineStr"/>
       <c r="O14" s="11" t="inlineStr">
         <is>
-          <t>ee1aed0</t>
+          <t>ee1aed0 | Released: Play 1.0.0+8 (published to everyone 2026-10-13; commit is in tag play-8)</t>
         </is>
       </c>
       <c r="P14" s="11" t="inlineStr">
@@ -2219,7 +2219,7 @@
       <c r="Q14" s="11" t="inlineStr"/>
       <c r="R14" s="11" t="inlineStr">
         <is>
-          <t>Also fixed: the Report sheet overflowed on short screens.</t>
+          <t>Also fixed: the Report sheet overflowed on short screens. | Status set to Released on 2026-10-14 from git: this commit is in the source of Play 1.0.0+8. Not yet verified by a person.</t>
         </is>
       </c>
     </row>
@@ -2342,13 +2342,13 @@
       <c r="L16" s="11" t="inlineStr"/>
       <c r="M16" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="N16" s="11" t="inlineStr"/>
       <c r="O16" s="11" t="inlineStr">
         <is>
-          <t>Oct 4 batch</t>
+          <t>Oct 4 batch | Released: Play 1.0.0+8 (published to everyone 2026-10-13; commit is in tag play-8)</t>
         </is>
       </c>
       <c r="P16" s="11" t="inlineStr">
@@ -2357,7 +2357,11 @@
         </is>
       </c>
       <c r="Q16" s="11" t="inlineStr"/>
-      <c r="R16" s="11" t="inlineStr"/>
+      <c r="R16" s="11" t="inlineStr">
+        <is>
+          <t>Status set to Released on 2026-10-14 from git: this commit is in the source of Play 1.0.0+8. Not yet verified by a person.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="n">
@@ -2408,13 +2412,13 @@
       <c r="L17" s="11" t="inlineStr"/>
       <c r="M17" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="N17" s="11" t="inlineStr"/>
       <c r="O17" s="11" t="inlineStr">
         <is>
-          <t>Oct 4 batch</t>
+          <t>Oct 4 batch | Released: Play 1.0.0+8 (published to everyone 2026-10-13; commit is in tag play-8)</t>
         </is>
       </c>
       <c r="P17" s="11" t="inlineStr">
@@ -2423,7 +2427,11 @@
         </is>
       </c>
       <c r="Q17" s="11" t="inlineStr"/>
-      <c r="R17" s="11" t="inlineStr"/>
+      <c r="R17" s="11" t="inlineStr">
+        <is>
+          <t>Status set to Released on 2026-10-14 from git: this commit is in the source of Play 1.0.0+8. Not yet verified by a person.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n">
@@ -2474,13 +2482,13 @@
       <c r="L18" s="11" t="inlineStr"/>
       <c r="M18" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="N18" s="11" t="inlineStr"/>
       <c r="O18" s="11" t="inlineStr">
         <is>
-          <t>Oct 4 batch</t>
+          <t>Oct 4 batch | Released: Play 1.0.0+8 (published to everyone 2026-10-13; commit is in tag play-8)</t>
         </is>
       </c>
       <c r="P18" s="11" t="inlineStr">
@@ -2489,7 +2497,11 @@
         </is>
       </c>
       <c r="Q18" s="11" t="inlineStr"/>
-      <c r="R18" s="11" t="inlineStr"/>
+      <c r="R18" s="11" t="inlineStr">
+        <is>
+          <t>Status set to Released on 2026-10-14 from git: this commit is in the source of Play 1.0.0+8. Not yet verified by a person.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="n">
@@ -3408,25 +3420,1881 @@
       <c r="L31" s="11" t="inlineStr"/>
       <c r="M31" s="11" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="N31" s="11" t="inlineStr"/>
-      <c r="O31" s="11" t="inlineStr"/>
+      <c r="O31" s="11" t="inlineStr">
+        <is>
+          <t>scripts/release/build_play_bundle.sh; close other Flutter / IDE windows first</t>
+        </is>
+      </c>
       <c r="P31" s="11" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="Q31" s="11" t="inlineStr"/>
+      <c r="Q31" s="11" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-13: the signed 1.0.0+8 bundle built and passed the script's checks (Gradle about 156 s)</t>
+        </is>
+      </c>
       <c r="R31" s="11" t="inlineStr">
         <is>
-          <t>1.0.0+8 bundle not built yet.</t>
+          <t>1.0.0+8 bundle not built yet. | Built successfully on 2026-10-13 09:56 IST.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>Games (Tulasi)</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>Improvement</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H32" s="11" t="inlineStr">
+        <is>
+          <t>Games from the Tulasi platform inside the app (Android only): the Games tab, a Games row on Home, and Games in the More menu of audio, video, host and PK rooms. A game opens in a panel at the bottom; the list, pictures and the Games switch update live; games can be hidden or shown from the panel; 18+ notice and date-of-birth rule; balance calls are handled by our backend.</t>
+        </is>
+      </c>
+      <c r="I32" s="11" t="inlineStr">
+        <is>
+          <t>Release controls &gt; Games ON; open the Games tab on an Android phone with 1.0.0+8.</t>
+        </is>
+      </c>
+      <c r="J32" s="11" t="inlineStr">
+        <is>
+          <t>Expected: the shown games open and play with the user's coins. Actual: works; 23 players and 14,056 successful balance calls on 13-14 Oct; the wallet ledger reconciles to the coin.</t>
+        </is>
+      </c>
+      <c r="K32" s="11" t="inlineStr">
+        <is>
+          <t>Android, Play build 1.0.0+8; Tulasi merchant 1503251, Singapore node</t>
+        </is>
+      </c>
+      <c r="L32" s="11" t="n"/>
+      <c r="M32" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="N32" s="11" t="n"/>
+      <c r="O32" s="11" t="inlineStr">
+        <is>
+          <t>1.0.0+8 (0d550ff); migrations 20261013100000 to 20261013140000; Edge function tulasi; panel main b37c27e</t>
+        </is>
+      </c>
+      <c r="P32" s="11" t="inlineStr">
+        <is>
+          <t>App build, Database migration, Edge function, Panel deploy</t>
+        </is>
+      </c>
+      <c r="Q32" s="11" t="inlineStr">
+        <is>
+          <t>Owner on the staging APK 2026-10-13; production play checked in the data by Claude 2026-10-14; the owner's own production round is still pending</t>
+        </is>
+      </c>
+      <c r="R32" s="11" t="inlineStr">
+        <is>
+          <t>Live since the Games switch was turned ON at 14:01 IST on 2026-10-13 with 10 of the 44 games shown. Android only; an iPhone shows 'coming soon'. Details: sabalive/docs/TULASI_GAMES.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>Games / live room</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H33" s="11" t="inlineStr">
+        <is>
+          <t>A game opened from an audio live showed half the game and a black block covering the live; the Games list stayed behind it and the live above was not usable.</t>
+        </is>
+      </c>
+      <c r="I33" s="11" t="inlineStr">
+        <is>
+          <t>Start an audio live &gt; More &gt; Games &gt; open a game.</t>
+        </is>
+      </c>
+      <c r="J33" s="11" t="inlineStr">
+        <is>
+          <t>Expected: a game panel at the bottom with the live visible and usable above it. Actual: a 90% tall sheet with a black top, the Games list still behind it.</t>
+        </is>
+      </c>
+      <c r="K33" s="11" t="inlineStr">
+        <is>
+          <t>Realme RMX1992 (Android), staging APK 1.0.0+8 of 2026-10-13</t>
+        </is>
+      </c>
+      <c r="L33" s="11" t="n"/>
+      <c r="M33" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="N33" s="11" t="n"/>
+      <c r="O33" s="11" t="inlineStr">
+        <is>
+          <t>1.0.0+8 (0d550ff): GamePanelRoute + showGamePanel; the panel height is read from the game page</t>
+        </is>
+      </c>
+      <c r="P33" s="11" t="inlineStr">
+        <is>
+          <t>App build</t>
+        </is>
+      </c>
+      <c r="Q33" s="11" t="inlineStr">
+        <is>
+          <t>Owner, staging APK built 07:11 IST 2026-10-13 ('fix is done'); not yet on the Play build</t>
+        </is>
+      </c>
+      <c r="R33" s="11" t="inlineStr">
+        <is>
+          <t>ROOT CAUSE: the games are Cocos canvases that keep the screen width and hang from the bottom, so extra height shows black; every game reports 750x1334 until its assets finish loading, so that value is ignored for 90 s. Measured: Teen Patti Gold, Dragon Tiger Battle, Lucky99 square; Greedy and Roulette 1.6x tall.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>Tulasi push (Sync Game List)</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>Build/Infra</t>
+        </is>
+      </c>
+      <c r="G34" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H34" s="11" t="inlineStr">
+        <is>
+          <t>Sync Game List in the Tulasi dashboard said 'Sync game list fail'. Two causes: our function copied every picture before answering (15 s), and decrypting the full 44-game push with pure-JavaScript RSA exceeded the Edge Function CPU limit (HTTP 546). FIX: answer first and copy pictures in the background; native RSA decryption; accept the platform's real payload (no status field, relative picture paths).</t>
+        </is>
+      </c>
+      <c r="I34" s="11" t="inlineStr">
+        <is>
+          <t>Tulasi dashboard &gt; Merchant Game Config &gt; Sync Game List &gt; Confirm.</t>
+        </is>
+      </c>
+      <c r="J34" s="11" t="inlineStr">
+        <is>
+          <t>Expected: success and the list in our database. Actual: fail, nothing written.</t>
+        </is>
+      </c>
+      <c r="K34" s="11" t="inlineStr">
+        <is>
+          <t>Supabase Edge Function tulasi (staging, then production)</t>
+        </is>
+      </c>
+      <c r="L34" s="11" t="n"/>
+      <c r="M34" s="11" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N34" s="11" t="n"/>
+      <c r="O34" s="11" t="inlineStr">
+        <is>
+          <t>tulasi function (commits up to 5771196); migration 20261013140000</t>
+        </is>
+      </c>
+      <c r="P34" s="11" t="inlineStr">
+        <is>
+          <t>Edge function, Database migration</t>
+        </is>
+      </c>
+      <c r="Q34" s="11" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-13: the dashboard said 'Sync game list success' on staging and then on production (44 games, 44 logos and banners copied to our storage)</t>
+        </is>
+      </c>
+      <c r="R34" s="11" t="inlineStr">
+        <is>
+          <t>The platform's Request Tester sends different fields from its documentation. A header x-decrypt tells which RSA path ran; x-config says why keys are unusable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D35" s="11" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>Games / limits</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>Policy</t>
+        </is>
+      </c>
+      <c r="G35" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H35" s="11" t="inlineStr">
+        <is>
+          <t>Players can bet up to 100,000 coins per bet and there is no daily loss or win cap. Overnight 23 players bet 13.8M coins and got back 10.6M; 6 of 23 lost more than 50,000 and some ended with almost no coins.</t>
+        </is>
+      </c>
+      <c r="I35" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J35" s="11" t="inlineStr">
+        <is>
+          <t>Suggested caps: largest bet 10,000, daily loss 50,000, daily win 200,000. Actual: 100,000 / none / none.</t>
+        </is>
+      </c>
+      <c r="K35" s="11" t="inlineStr">
+        <is>
+          <t>Production, game_config</t>
+        </is>
+      </c>
+      <c r="L35" s="11" t="n"/>
+      <c r="M35" s="11" t="inlineStr">
+        <is>
+          <t>Won't fix</t>
+        </is>
+      </c>
+      <c r="N35" s="11" t="n"/>
+      <c r="O35" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P35" s="11" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="Q35" s="11" t="inlineStr">
+        <is>
+          <t>Owner decision 2026-10-14: keep the existing numbers</t>
+        </is>
+      </c>
+      <c r="R35" s="11" t="inlineStr">
+        <is>
+          <t>Revisit with more data. The limits can be changed at any time on the panel's Games page and apply to the next bet. Other protections stay: 18+ rule, payout cap (100x the bets on that game in 15 minutes), refusal of late or duplicate calls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>Play Console / games</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="inlineStr">
+        <is>
+          <t>Policy</t>
+        </is>
+      </c>
+      <c r="G36" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H36" s="11" t="inlineStr">
+        <is>
+          <t>Confirm that the Play Console content rating and declarations describe the games (simulated casino-style games with purchasable coins, 18+ audience) and that the reviewer notes say the feature is included and turned on from the panel. The games were switched ON for everyone on 2026-10-13 after 1.0.0+8 was approved.</t>
+        </is>
+      </c>
+      <c r="I36" s="11" t="inlineStr">
+        <is>
+          <t>Play Console &gt; App content.</t>
+        </is>
+      </c>
+      <c r="J36" s="11" t="inlineStr">
+        <is>
+          <t>Expected: declarations match the live features. Actual: not confirmed.</t>
+        </is>
+      </c>
+      <c r="K36" s="11" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="L36" s="11" t="n"/>
+      <c r="M36" s="11" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="N36" s="11" t="n"/>
+      <c r="O36" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P36" s="11" t="inlineStr">
+        <is>
+          <t>Store / console action</t>
+        </is>
+      </c>
+      <c r="Q36" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R36" s="11" t="inlineStr">
+        <is>
+          <t>The Tulasi guide says outcomes can be adjusted (platform commission, interventions, robot players); the in-app notice says so. A policy strike could affect the whole app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D37" s="11" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="E37" s="11" t="inlineStr">
+        <is>
+          <t>Tulasi account</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
+          <t>Build/Infra</t>
+        </is>
+      </c>
+      <c r="G37" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H37" s="11" t="inlineStr">
+        <is>
+          <t>The Tulasi dashboard shows an account Expire Date of 2026-11-22 14:00 (UTC+8). The games stop when it passes unless Tulasi renews it.</t>
+        </is>
+      </c>
+      <c r="I37" s="11" t="inlineStr">
+        <is>
+          <t>Tulasi dashboard, top of the first page.</t>
+        </is>
+      </c>
+      <c r="J37" s="11" t="inlineStr">
+        <is>
+          <t>Expected: renewed before the date. Actual: not yet.</t>
+        </is>
+      </c>
+      <c r="K37" s="11" t="inlineStr">
+        <is>
+          <t>Tulasi dashboard</t>
+        </is>
+      </c>
+      <c r="L37" s="11" t="n"/>
+      <c r="M37" s="11" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="N37" s="11" t="n"/>
+      <c r="O37" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P37" s="11" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="Q37" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R37" s="11" t="inlineStr">
+        <is>
+          <t>Ask Tulasi about renewal, fees, a failure code for refused calls, and whether Sync Game List can be automatic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>Security / credentials</t>
+        </is>
+      </c>
+      <c r="F38" s="10" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G38" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H38" s="11" t="inlineStr">
+        <is>
+          <t>The Tulasi dashboard password was pasted into the chat early in the work, and the first lines of the private-key box were visible in screenshots while setting the keys on staging. Change the password. Rotate the keys with Reset only together with re-setting the secrets on BOTH Supabase projects.</t>
+        </is>
+      </c>
+      <c r="I38" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J38" s="11" t="inlineStr">
+        <is>
+          <t>Expected: no credential in a chat. Actual: shared once.</t>
+        </is>
+      </c>
+      <c r="K38" s="11" t="inlineStr">
+        <is>
+          <t>Tulasi dashboard</t>
+        </is>
+      </c>
+      <c r="L38" s="11" t="n"/>
+      <c r="M38" s="11" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="N38" s="11" t="n"/>
+      <c r="O38" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P38" s="11" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="Q38" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R38" s="11" t="inlineStr">
+        <is>
+          <t>The same keys are set on staging and production (one merchant).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>Games on iPhone</t>
+        </is>
+      </c>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>Improvement</t>
+        </is>
+      </c>
+      <c r="G39" s="10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H39" s="11" t="inlineStr">
+        <is>
+          <t>iPhones show 'coming soon': the games are Android only until the store and legal review for Apple is settled.</t>
+        </is>
+      </c>
+      <c r="I39" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J39" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K39" s="11" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="L39" s="11" t="n"/>
+      <c r="M39" s="11" t="inlineStr">
+        <is>
+          <t>Needs decision</t>
+        </is>
+      </c>
+      <c r="N39" s="11" t="n"/>
+      <c r="O39" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P39" s="11" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="Q39" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R39" s="11" t="inlineStr">
+        <is>
+          <t>Apple 5.3 / 4.7 rules for gambling-style content need a separate review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>Backend (Supabase)</t>
+        </is>
+      </c>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>Build/Infra</t>
+        </is>
+      </c>
+      <c r="G40" s="10" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="H40" s="11" t="inlineStr">
+        <is>
+          <t>Production stalled repeatedly on 13 Oct: background jobs failed to start from 13:43, a 2.5 minute outage at 13:49 after the owner restarted the project, more stalls at 14:05, 14:13, 14:16 and 14:18. Traffic was small (about 8 requests per second, about 10 users): no attack was found. The machine was starved.</t>
+        </is>
+      </c>
+      <c r="I40" s="11" t="inlineStr">
+        <is>
+          <t>scripts/prod/healthcheck.sh: 'could not query the database' or a status call of several seconds.</t>
+        </is>
+      </c>
+      <c r="J40" s="11" t="inlineStr">
+        <is>
+          <t>Expected: status call under 1 s. Actual: up to 7 s and 521/502 errors.</t>
+        </is>
+      </c>
+      <c r="K40" s="11" t="inlineStr">
+        <is>
+          <t>Supabase production, Micro-class compute</t>
+        </is>
+      </c>
+      <c r="L40" s="11" t="n"/>
+      <c r="M40" s="11" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N40" s="11" t="n"/>
+      <c r="O40" s="11" t="inlineStr">
+        <is>
+          <t>Compute upgraded by the owner at 14:27 IST on 2026-10-13</t>
+        </is>
+      </c>
+      <c r="P40" s="11" t="inlineStr">
+        <is>
+          <t>Store / console action</t>
+        </is>
+      </c>
+      <c r="Q40" s="11" t="inlineStr">
+        <is>
+          <t>Claude, 2026-10-14 06:40: zero failed jobs for 16 hours; the gate function 7.4 ms to 0.09 ms; CPU test 47 ms (idle staging 50 ms)</t>
+        </is>
+      </c>
+      <c r="R40" s="11" t="inlineStr">
+        <is>
+          <t>Evidence and queries are in HANDOFF.md. Do not restart to fix this. Maintenance ended at 13:26 and 1.0.0+8 reached everyone at once the same afternoon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D41" s="11" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="E41" s="11" t="inlineStr">
+        <is>
+          <t>Release scripts</t>
+        </is>
+      </c>
+      <c r="F41" s="10" t="inlineStr">
+        <is>
+          <t>Build/Infra</t>
+        </is>
+      </c>
+      <c r="G41" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H41" s="11" t="inlineStr">
+        <is>
+          <t>In a normal terminal 'supabase db query -o json' prints a plain list, but when an agent runs it the result is wrapped in {rows}. The health check, smoke test, backup and staging scripts only understood the wrapped form, so in the owner's terminal every migration stopped at 'could not query the database'. FIX: all scripts accept both; a timed-out call is retried 3 times.</t>
+        </is>
+      </c>
+      <c r="I41" s="11" t="inlineStr">
+        <is>
+          <t>Run scripts/prod/healthcheck.sh in a normal terminal.</t>
+        </is>
+      </c>
+      <c r="J41" s="11" t="inlineStr">
+        <is>
+          <t>Expected: checks run. Actual: FAIL could not query the database.</t>
+        </is>
+      </c>
+      <c r="K41" s="11" t="inlineStr">
+        <is>
+          <t>macOS terminal, Supabase CLI 2.101</t>
+        </is>
+      </c>
+      <c r="L41" s="11" t="n"/>
+      <c r="M41" s="11" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="N41" s="11" t="n"/>
+      <c r="O41" s="11" t="inlineStr">
+        <is>
+          <t>e484cb6, 5d624c9 (sabalive, now on main)</t>
+        </is>
+      </c>
+      <c r="P41" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="Q41" s="11" t="inlineStr">
+        <is>
+          <t>Owner's terminal, 2026-10-13: 16 migrations ran with every check passing</t>
+        </is>
+      </c>
+      <c r="R41" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>Release 1.0.0+8</t>
+        </is>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>Build/Infra</t>
+        </is>
+      </c>
+      <c r="G42" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H42" s="11" t="inlineStr">
+        <is>
+          <t>Bundle 1.0.0+8 was built with scripts/release/build_play_bundle.sh (signed with the release key, only the production Supabase address inside, permissions identical to 1.0.0+7), approved by Google and published to everyone at once (no staged rollout) on 2026-10-13.</t>
+        </is>
+      </c>
+      <c r="I42" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J42" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K42" s="11" t="inlineStr">
+        <is>
+          <t>Google Play</t>
+        </is>
+      </c>
+      <c r="L42" s="11" t="n"/>
+      <c r="M42" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="N42" s="11" t="n"/>
+      <c r="O42" s="11" t="inlineStr">
+        <is>
+          <t>1.0.0+8 = tag play-8 (0d550ff)</t>
+        </is>
+      </c>
+      <c r="P42" s="11" t="inlineStr">
+        <is>
+          <t>Store / console action</t>
+        </is>
+      </c>
+      <c r="Q42" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R42" s="11" t="inlineStr">
+        <is>
+          <t>Tags: play-live = 1.0.0+7 (rollback anchor), play-8, prod-20261013 (app 1dad240, panel b37c27e). The database was upgraded first (16 migrations under maintenance) so new apps found everything they need.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D43" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E43" s="11" t="inlineStr">
+        <is>
+          <t>Live rooms: moderation</t>
+        </is>
+      </c>
+      <c r="F43" s="10" t="inlineStr">
+        <is>
+          <t>Improvement</t>
+        </is>
+      </c>
+      <c r="G43" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H43" s="11" t="inlineStr">
+        <is>
+          <t>Room admins (the host adds up to 5), kick, ban and ban text, report, in audio and video lives; the moderation lists update live.</t>
+        </is>
+      </c>
+      <c r="I43" s="11" t="inlineStr">
+        <is>
+          <t>Host Tools &gt; Room admins; tap a person &gt; Kick / Ban / Ban text.</t>
+        </is>
+      </c>
+      <c r="J43" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K43" s="11" t="inlineStr">
+        <is>
+          <t>Android, 1.0.0+8</t>
+        </is>
+      </c>
+      <c r="L43" s="11" t="n"/>
+      <c r="M43" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="N43" s="11" t="n"/>
+      <c r="O43" s="11" t="inlineStr">
+        <is>
+          <t>1.0.0+8; migration 20261010100000</t>
+        </is>
+      </c>
+      <c r="P43" s="11" t="inlineStr">
+        <is>
+          <t>App build, Database migration</t>
+        </is>
+      </c>
+      <c r="Q43" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R43" s="11" t="inlineStr">
+        <is>
+          <t>The options are hidden in the app on a database without the migration; applied on production 2026-10-13.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D44" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E44" s="11" t="inlineStr">
+        <is>
+          <t>Audio and video seats</t>
+        </is>
+      </c>
+      <c r="F44" s="10" t="inlineStr">
+        <is>
+          <t>Improvement</t>
+        </is>
+      </c>
+      <c r="G44" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H44" s="11" t="inlineStr">
+        <is>
+          <t>Audio seats 4 per row and 4 to 16 seats; video guest seats in a right-hand column; seat glitch hardening (a seat re-read that raced a Realtime change could overwrite the screen with an old list).</t>
+        </is>
+      </c>
+      <c r="I44" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J44" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K44" s="11" t="inlineStr">
+        <is>
+          <t>Android, 1.0.0+8</t>
+        </is>
+      </c>
+      <c r="L44" s="11" t="n"/>
+      <c r="M44" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="N44" s="11" t="n"/>
+      <c r="O44" s="11" t="inlineStr">
+        <is>
+          <t>1.0.0+8 (0d550ff)</t>
+        </is>
+      </c>
+      <c r="P44" s="11" t="inlineStr">
+        <is>
+          <t>App build</t>
+        </is>
+      </c>
+      <c r="Q44" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R44" s="11" t="inlineStr">
+        <is>
+          <t>The owner's report gave no detail: the likely causes were hardened; not confirmed on devices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C45" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D45" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E45" s="11" t="inlineStr">
+        <is>
+          <t>Seat speaking indicator</t>
+        </is>
+      </c>
+      <c r="F45" s="10" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="G45" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H45" s="11" t="inlineStr">
+        <is>
+          <t>Voice waves did not show when OTHER people spoke. FIX: remote speakers light a seat at volume 10 or more (own microphone 25); an unknown speaking id triggers a throttled seat re-read; wave colours per person, host always green.</t>
+        </is>
+      </c>
+      <c r="I45" s="11" t="inlineStr">
+        <is>
+          <t>Two phones in an audio live; one speaks.</t>
+        </is>
+      </c>
+      <c r="J45" s="11" t="inlineStr">
+        <is>
+          <t>Expected: the speaker's seat shows waves on both phones. Actual: only the speaker's own.</t>
+        </is>
+      </c>
+      <c r="K45" s="11" t="inlineStr">
+        <is>
+          <t>Android, 1.0.0+8</t>
+        </is>
+      </c>
+      <c r="L45" s="11" t="n"/>
+      <c r="M45" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="N45" s="11" t="n"/>
+      <c r="O45" s="11" t="inlineStr">
+        <is>
+          <t>1.0.0+8 (0d550ff)</t>
+        </is>
+      </c>
+      <c r="P45" s="11" t="inlineStr">
+        <is>
+          <t>App build</t>
+        </is>
+      </c>
+      <c r="Q45" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R45" s="11" t="inlineStr">
+        <is>
+          <t>Could not be reproduced from code; not confirmed on devices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E46" s="11" t="inlineStr">
+        <is>
+          <t>Live chat / emotes</t>
+        </is>
+      </c>
+      <c r="F46" s="10" t="inlineStr">
+        <is>
+          <t>Improvement</t>
+        </is>
+      </c>
+      <c r="G46" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H46" s="11" t="inlineStr">
+        <is>
+          <t>Emoji renamed Emotes: an emote plays over the sender's picture circle (slower: grows and fades), 53 more emotes; the panel page is Emotes &amp; GIFs.</t>
+        </is>
+      </c>
+      <c r="I46" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J46" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K46" s="11" t="inlineStr">
+        <is>
+          <t>Android, 1.0.0+8</t>
+        </is>
+      </c>
+      <c r="L46" s="11" t="n"/>
+      <c r="M46" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="N46" s="11" t="n"/>
+      <c r="O46" s="11" t="inlineStr">
+        <is>
+          <t>1.0.0+8; migration 20261012110000; panel part 1</t>
+        </is>
+      </c>
+      <c r="P46" s="11" t="inlineStr">
+        <is>
+          <t>App build, Database migration, Panel deploy</t>
+        </is>
+      </c>
+      <c r="Q46" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R46" s="11" t="inlineStr">
+        <is>
+          <t>Production now has 64 emotes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="C47" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D47" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E47" s="11" t="inlineStr">
+        <is>
+          <t>Level banner / entry effect</t>
+        </is>
+      </c>
+      <c r="F47" s="10" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="G47" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H47" s="11" t="inlineStr">
+        <is>
+          <t>The level join banner was too fast, used the wrong picture, was missing for some viewers and showed twice. FIX: slower (5.2 s hold), uses the charm level picture, the joiner's own banner plays at once, and the entry is claimed before any wait so it plays once.</t>
+        </is>
+      </c>
+      <c r="I47" s="11" t="inlineStr">
+        <is>
+          <t>Join a live that has viewers.</t>
+        </is>
+      </c>
+      <c r="J47" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K47" s="11" t="inlineStr">
+        <is>
+          <t>Android, 1.0.0+8</t>
+        </is>
+      </c>
+      <c r="L47" s="11" t="n"/>
+      <c r="M47" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="N47" s="11" t="n"/>
+      <c r="O47" s="11" t="inlineStr">
+        <is>
+          <t>1.0.0+8 (0d550ff)</t>
+        </is>
+      </c>
+      <c r="P47" s="11" t="inlineStr">
+        <is>
+          <t>App build</t>
+        </is>
+      </c>
+      <c r="Q47" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R47" s="11" t="inlineStr">
+        <is>
+          <t>Seeing OTHER people's arrivals still depends on Realtime; not confirmed on devices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E48" s="11" t="inlineStr">
+        <is>
+          <t>Avatar frames</t>
+        </is>
+      </c>
+      <c r="F48" s="10" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="G48" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H48" s="11" t="inlineStr">
+        <is>
+          <t>Frames overlapped faces and spilled out of seats and the profile. FIX: the size now includes the frame, the picture is drawn in front, no frame below 40 px, seats reserve one square.</t>
+        </is>
+      </c>
+      <c r="I48" s="11" t="inlineStr">
+        <is>
+          <t>Look at seats and profiles with a frame.</t>
+        </is>
+      </c>
+      <c r="J48" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K48" s="11" t="inlineStr">
+        <is>
+          <t>Android, 1.0.0+8</t>
+        </is>
+      </c>
+      <c r="L48" s="11" t="n"/>
+      <c r="M48" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="N48" s="11" t="n"/>
+      <c r="O48" s="11" t="inlineStr">
+        <is>
+          <t>1.0.0+8 (0d550ff)</t>
+        </is>
+      </c>
+      <c r="P48" s="11" t="inlineStr">
+        <is>
+          <t>App build</t>
+        </is>
+      </c>
+      <c r="Q48" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R48" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C49" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E49" s="11" t="inlineStr">
+        <is>
+          <t>Lucky Box</t>
+        </is>
+      </c>
+      <c r="F49" s="10" t="inlineStr">
+        <is>
+          <t>Improvement</t>
+        </is>
+      </c>
+      <c r="G49" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H49" s="11" t="inlineStr">
+        <is>
+          <t>The Lucky Box timer is shown to the host only (not viewers); one reward per host per 24 hours (cooldown set in the panel).</t>
+        </is>
+      </c>
+      <c r="I49" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J49" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K49" s="11" t="inlineStr">
+        <is>
+          <t>Android, 1.0.0+8</t>
+        </is>
+      </c>
+      <c r="L49" s="11" t="n"/>
+      <c r="M49" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="N49" s="11" t="n"/>
+      <c r="O49" s="11" t="inlineStr">
+        <is>
+          <t>1.0.0+8; migration 20261010090000; panel part 2</t>
+        </is>
+      </c>
+      <c r="P49" s="11" t="inlineStr">
+        <is>
+          <t>App build, Database migration, Panel deploy</t>
+        </is>
+      </c>
+      <c r="Q49" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R49" s="11" t="inlineStr">
+        <is>
+          <t>Applied on production 2026-10-13.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E50" s="11" t="inlineStr">
+        <is>
+          <t>Screen protection</t>
+        </is>
+      </c>
+      <c r="F50" s="10" t="inlineStr">
+        <is>
+          <t>Improvement</t>
+        </is>
+      </c>
+      <c r="G50" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H50" s="11" t="inlineStr">
+        <is>
+          <t>Android shows a black picture to screenshots, screen recording, casting and the recent-apps list when the panel switch is on (default off).</t>
+        </is>
+      </c>
+      <c r="I50" s="11" t="inlineStr">
+        <is>
+          <t>Release controls &gt; Block screenshots and screen recording ON.</t>
+        </is>
+      </c>
+      <c r="J50" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K50" s="11" t="inlineStr">
+        <is>
+          <t>Android, 1.0.0+8</t>
+        </is>
+      </c>
+      <c r="L50" s="11" t="n"/>
+      <c r="M50" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="N50" s="11" t="n"/>
+      <c r="O50" s="11" t="inlineStr">
+        <is>
+          <t>1.0.0+8; panel part 1</t>
+        </is>
+      </c>
+      <c r="P50" s="11" t="inlineStr">
+        <is>
+          <t>App build, Panel deploy</t>
+        </is>
+      </c>
+      <c r="Q50" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R50" s="11" t="inlineStr">
+        <is>
+          <t>The switch is currently OFF. iPhones cannot block screenshots.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D51" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E51" s="11" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="F51" s="10" t="inlineStr">
+        <is>
+          <t>Improvement</t>
+        </is>
+      </c>
+      <c r="G51" s="10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H51" s="11" t="inlineStr">
+        <is>
+          <t>Social login shown as two full-width banners, Google and Apple.</t>
+        </is>
+      </c>
+      <c r="I51" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J51" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K51" s="11" t="inlineStr">
+        <is>
+          <t>Android and iOS, 1.0.0+8</t>
+        </is>
+      </c>
+      <c r="L51" s="11" t="n"/>
+      <c r="M51" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="N51" s="11" t="n"/>
+      <c r="O51" s="11" t="inlineStr">
+        <is>
+          <t>1.0.0+8 (0d550ff)</t>
+        </is>
+      </c>
+      <c r="P51" s="11" t="inlineStr">
+        <is>
+          <t>App build</t>
+        </is>
+      </c>
+      <c r="Q51" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R51" s="11" t="inlineStr">
+        <is>
+          <t>Apple's guidelines ask for 'Sign in with Apple' wording: check at review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="C52" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D52" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E52" s="11" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
+      <c r="F52" s="10" t="inlineStr">
+        <is>
+          <t>Improvement</t>
+        </is>
+      </c>
+      <c r="G52" s="10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H52" s="11" t="inlineStr">
+        <is>
+          <t>Garage tab removed (Store tabs: Frame, Lucky ID, Entry, Room Skin); room skin picker; theme and branding colours come from the panel.</t>
+        </is>
+      </c>
+      <c r="I52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K52" s="11" t="inlineStr">
+        <is>
+          <t>Android, 1.0.0+8</t>
+        </is>
+      </c>
+      <c r="L52" s="11" t="n"/>
+      <c r="M52" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="N52" s="11" t="n"/>
+      <c r="O52" s="11" t="inlineStr">
+        <is>
+          <t>1.0.0+8 (0d550ff)</t>
+        </is>
+      </c>
+      <c r="P52" s="11" t="inlineStr">
+        <is>
+          <t>App build</t>
+        </is>
+      </c>
+      <c r="Q52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C53" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D53" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E53" s="11" t="inlineStr">
+        <is>
+          <t>Live gifts and rooms</t>
+        </is>
+      </c>
+      <c r="F53" s="10" t="inlineStr">
+        <is>
+          <t>Improvement</t>
+        </is>
+      </c>
+      <c r="G53" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H53" s="11" t="inlineStr">
+        <is>
+          <t>Send a gift to All (one gift to everyone in the room); effect play speed and sound per effect; leaving a live frees the seat at once and silent viewers are swept after 75 s.</t>
+        </is>
+      </c>
+      <c r="I53" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J53" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K53" s="11" t="inlineStr">
+        <is>
+          <t>Android, 1.0.0+8</t>
+        </is>
+      </c>
+      <c r="L53" s="11" t="n"/>
+      <c r="M53" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="N53" s="11" t="n"/>
+      <c r="O53" s="11" t="inlineStr">
+        <is>
+          <t>1.0.0+8; migrations 20261009100000, 20261009110000, 20261009120000</t>
+        </is>
+      </c>
+      <c r="P53" s="11" t="inlineStr">
+        <is>
+          <t>App build, Database migration, Panel deploy</t>
+        </is>
+      </c>
+      <c r="Q53" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R53" s="11" t="inlineStr">
+        <is>
+          <t>Applied on production 2026-10-13.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R31"/>
+  <autoFilter ref="A1:R53"/>
   <conditionalFormatting sqref="G2:G400">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Critical"</formula>
@@ -3500,7 +5368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S18"/>
+  <dimension ref="A1:S24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3671,13 +5539,13 @@
       <c r="M2" s="11" t="inlineStr"/>
       <c r="N2" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="O2" s="11" t="inlineStr"/>
       <c r="P2" s="11" t="inlineStr">
         <is>
-          <t>Oct 3</t>
+          <t>Oct 3 | Released: live on the admin panel (main b37c27e, 2026-10-13); its database part is applied on production</t>
         </is>
       </c>
       <c r="Q2" s="11" t="inlineStr">
@@ -3688,7 +5556,7 @@
       <c r="R2" s="11" t="inlineStr"/>
       <c r="S2" s="11" t="inlineStr">
         <is>
-          <t>Edge function ghost-admin deployed.</t>
+          <t>Edge function ghost-admin deployed. | Status set to Released on 2026-10-14: the panel deploys from main, which now contains this change. Not yet verified by a person.</t>
         </is>
       </c>
     </row>
@@ -3742,13 +5610,13 @@
       <c r="M3" s="11" t="inlineStr"/>
       <c r="N3" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="O3" s="11" t="inlineStr"/>
       <c r="P3" s="11" t="inlineStr">
         <is>
-          <t>Oct 3</t>
+          <t>Oct 3 | Released: live on the admin panel (main b37c27e, 2026-10-13); its database part is applied on production</t>
         </is>
       </c>
       <c r="Q3" s="11" t="inlineStr">
@@ -3757,7 +5625,11 @@
         </is>
       </c>
       <c r="R3" s="11" t="inlineStr"/>
-      <c r="S3" s="11" t="inlineStr"/>
+      <c r="S3" s="11" t="inlineStr">
+        <is>
+          <t>Status set to Released on 2026-10-14: the panel deploys from main, which now contains this change. Not yet verified by a person.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="n">
@@ -3809,13 +5681,13 @@
       <c r="M4" s="11" t="inlineStr"/>
       <c r="N4" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="O4" s="11" t="inlineStr"/>
       <c r="P4" s="11" t="inlineStr">
         <is>
-          <t>Oct 4 sync batch</t>
+          <t>Oct 4 sync batch | Released: live on the admin panel (main b37c27e, 2026-10-13); its database part is applied on production</t>
         </is>
       </c>
       <c r="Q4" s="11" t="inlineStr">
@@ -3824,7 +5696,11 @@
         </is>
       </c>
       <c r="R4" s="11" t="inlineStr"/>
-      <c r="S4" s="11" t="inlineStr"/>
+      <c r="S4" s="11" t="inlineStr">
+        <is>
+          <t>Status set to Released on 2026-10-14: the panel deploys from main, which now contains this change. Not yet verified by a person.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="n">
@@ -3876,13 +5752,13 @@
       <c r="M5" s="11" t="inlineStr"/>
       <c r="N5" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="O5" s="11" t="inlineStr"/>
       <c r="P5" s="11" t="inlineStr">
         <is>
-          <t>Oct 4 sync batch</t>
+          <t>Oct 4 sync batch | Released: live on the admin panel (main b37c27e, 2026-10-13); its database part is applied on production</t>
         </is>
       </c>
       <c r="Q5" s="11" t="inlineStr">
@@ -3891,7 +5767,11 @@
         </is>
       </c>
       <c r="R5" s="11" t="inlineStr"/>
-      <c r="S5" s="11" t="inlineStr"/>
+      <c r="S5" s="11" t="inlineStr">
+        <is>
+          <t>Status set to Released on 2026-10-14: the panel deploys from main, which now contains this change. Not yet verified by a person.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="n">
@@ -3943,13 +5823,13 @@
       <c r="M6" s="11" t="inlineStr"/>
       <c r="N6" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="O6" s="11" t="inlineStr"/>
       <c r="P6" s="11" t="inlineStr">
         <is>
-          <t>Oct 4 sync batch</t>
+          <t>Oct 4 sync batch | Released: live on the admin panel (main b37c27e, 2026-10-13); its database part is applied on production</t>
         </is>
       </c>
       <c r="Q6" s="11" t="inlineStr">
@@ -3958,7 +5838,11 @@
         </is>
       </c>
       <c r="R6" s="11" t="inlineStr"/>
-      <c r="S6" s="11" t="inlineStr"/>
+      <c r="S6" s="11" t="inlineStr">
+        <is>
+          <t>Status set to Released on 2026-10-14: the panel deploys from main, which now contains this change. Not yet verified by a person.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="n">
@@ -4010,13 +5894,13 @@
       <c r="M7" s="11" t="inlineStr"/>
       <c r="N7" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="O7" s="11" t="inlineStr"/>
       <c r="P7" s="11" t="inlineStr">
         <is>
-          <t>416ac77 / migration 20261005090000</t>
+          <t>416ac77 / migration 20261005090000 | Released: live on the admin panel (main b37c27e, 2026-10-13); its database part is applied on production</t>
         </is>
       </c>
       <c r="Q7" s="11" t="inlineStr">
@@ -4027,7 +5911,7 @@
       <c r="R7" s="11" t="inlineStr"/>
       <c r="S7" s="11" t="inlineStr">
         <is>
-          <t>Migration already applied by hand before the push; now recorded.</t>
+          <t>Migration already applied by hand before the push; now recorded. | Status set to Released on 2026-10-14: the panel deploys from main, which now contains this change. Not yet verified by a person.</t>
         </is>
       </c>
     </row>
@@ -4081,13 +5965,13 @@
       <c r="M8" s="11" t="inlineStr"/>
       <c r="N8" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="O8" s="11" t="inlineStr"/>
       <c r="P8" s="11" t="inlineStr">
         <is>
-          <t>Oct 4 sync batch</t>
+          <t>Oct 4 sync batch | Released: live on the admin panel (main b37c27e, 2026-10-13); its database part is applied on production</t>
         </is>
       </c>
       <c r="Q8" s="11" t="inlineStr">
@@ -4096,7 +5980,11 @@
         </is>
       </c>
       <c r="R8" s="11" t="inlineStr"/>
-      <c r="S8" s="11" t="inlineStr"/>
+      <c r="S8" s="11" t="inlineStr">
+        <is>
+          <t>Status set to Released on 2026-10-14: the panel deploys from main, which now contains this change. Not yet verified by a person.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="n">
@@ -4148,13 +6036,13 @@
       <c r="M9" s="11" t="inlineStr"/>
       <c r="N9" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="O9" s="11" t="inlineStr"/>
       <c r="P9" s="11" t="inlineStr">
         <is>
-          <t>Oct 4 sync batch</t>
+          <t>Oct 4 sync batch | Released: live on the admin panel (main b37c27e, 2026-10-13); its database part is applied on production</t>
         </is>
       </c>
       <c r="Q9" s="11" t="inlineStr">
@@ -4163,7 +6051,11 @@
         </is>
       </c>
       <c r="R9" s="11" t="inlineStr"/>
-      <c r="S9" s="11" t="inlineStr"/>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>Status set to Released on 2026-10-14: the panel deploys from main, which now contains this change. Not yet verified by a person.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="n">
@@ -4219,13 +6111,13 @@
       <c r="M10" s="11" t="inlineStr"/>
       <c r="N10" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="O10" s="11" t="inlineStr"/>
       <c r="P10" s="11" t="inlineStr">
         <is>
-          <t>7bdd076, 4ef891c, f213e62; migrations 20261005120000 and 140000</t>
+          <t>7bdd076, 4ef891c, f213e62; migrations 20261005120000 and 140000 | Released: live on the admin panel (main b37c27e, 2026-10-13); its database part is applied on production</t>
         </is>
       </c>
       <c r="Q10" s="11" t="inlineStr">
@@ -4236,7 +6128,7 @@
       <c r="R10" s="11" t="inlineStr"/>
       <c r="S10" s="11" t="inlineStr">
         <is>
-          <t>Migrations recorded in prod on 2026-10-06.</t>
+          <t>Migrations recorded in prod on 2026-10-06. | Status set to Released on 2026-10-14: the panel deploys from main, which now contains this change. Not yet verified by a person.</t>
         </is>
       </c>
     </row>
@@ -4294,13 +6186,13 @@
       <c r="M11" s="11" t="inlineStr"/>
       <c r="N11" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="O11" s="11" t="inlineStr"/>
       <c r="P11" s="11" t="inlineStr">
         <is>
-          <t>e74cc9e; migration 20261005160000</t>
+          <t>e74cc9e; migration 20261005160000 | Released: live on the admin panel (main b37c27e, 2026-10-13); its database part is applied on production</t>
         </is>
       </c>
       <c r="Q11" s="11" t="inlineStr">
@@ -4309,7 +6201,11 @@
         </is>
       </c>
       <c r="R11" s="11" t="inlineStr"/>
-      <c r="S11" s="11" t="inlineStr"/>
+      <c r="S11" s="11" t="inlineStr">
+        <is>
+          <t>Status set to Released on 2026-10-14: the panel deploys from main, which now contains this change. Not yet verified by a person.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="n">
@@ -4365,13 +6261,13 @@
       <c r="M12" s="11" t="inlineStr"/>
       <c r="N12" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="O12" s="11" t="inlineStr"/>
       <c r="P12" s="11" t="inlineStr">
         <is>
-          <t>05062b8, a4f31c3</t>
+          <t>05062b8, a4f31c3 | Released: live on the admin panel (main b37c27e, 2026-10-13); its database part is applied on production</t>
         </is>
       </c>
       <c r="Q12" s="11" t="inlineStr">
@@ -4380,7 +6276,11 @@
         </is>
       </c>
       <c r="R12" s="11" t="inlineStr"/>
-      <c r="S12" s="11" t="inlineStr"/>
+      <c r="S12" s="11" t="inlineStr">
+        <is>
+          <t>Status set to Released on 2026-10-14: the panel deploys from main, which now contains this change. Not yet verified by a person.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="n">
@@ -4436,13 +6336,13 @@
       <c r="M13" s="11" t="inlineStr"/>
       <c r="N13" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="O13" s="11" t="inlineStr"/>
       <c r="P13" s="11" t="inlineStr">
         <is>
-          <t>0c78788</t>
+          <t>0c78788 | Released: live on the admin panel (main b37c27e, 2026-10-13); its database part is applied on production</t>
         </is>
       </c>
       <c r="Q13" s="11" t="inlineStr">
@@ -4451,7 +6351,11 @@
         </is>
       </c>
       <c r="R13" s="11" t="inlineStr"/>
-      <c r="S13" s="11" t="inlineStr"/>
+      <c r="S13" s="11" t="inlineStr">
+        <is>
+          <t>Status set to Released on 2026-10-14: the panel deploys from main, which now contains this change. Not yet verified by a person.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="n">
@@ -4507,13 +6411,13 @@
       <c r="M14" s="11" t="inlineStr"/>
       <c r="N14" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="O14" s="11" t="inlineStr"/>
       <c r="P14" s="11" t="inlineStr">
         <is>
-          <t>cf4d71e</t>
+          <t>cf4d71e | Released: live on the admin panel (main b37c27e, 2026-10-13); its database part is applied on production</t>
         </is>
       </c>
       <c r="Q14" s="11" t="inlineStr">
@@ -4522,7 +6426,11 @@
         </is>
       </c>
       <c r="R14" s="11" t="inlineStr"/>
-      <c r="S14" s="11" t="inlineStr"/>
+      <c r="S14" s="11" t="inlineStr">
+        <is>
+          <t>Status set to Released on 2026-10-14: the panel deploys from main, which now contains this change. Not yet verified by a person.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="n">
@@ -4578,13 +6486,13 @@
       <c r="M15" s="11" t="inlineStr"/>
       <c r="N15" s="11" t="inlineStr">
         <is>
-          <t>Fixed (in code)</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="O15" s="11" t="inlineStr"/>
       <c r="P15" s="11" t="inlineStr">
         <is>
-          <t>15be4f6; migration 20261005200000</t>
+          <t>15be4f6; migration 20261005200000 | Released: live on the admin panel (main b37c27e, 2026-10-13); its database part is applied on production</t>
         </is>
       </c>
       <c r="Q15" s="11" t="inlineStr">
@@ -4595,7 +6503,7 @@
       <c r="R15" s="11" t="inlineStr"/>
       <c r="S15" s="11" t="inlineStr">
         <is>
-          <t>Policy already existed in prod before the push.</t>
+          <t>Policy already existed in prod before the push. | Status set to Released on 2026-10-14: the panel deploys from main, which now contains this change. Not yet verified by a person.</t>
         </is>
       </c>
     </row>
@@ -4804,12 +6712,498 @@
       <c r="R18" s="11" t="inlineStr"/>
       <c r="S18" s="11" t="inlineStr">
         <is>
-          <t>Part of the production-safety work.</t>
+          <t>Part of the production-safety work. | The Release controls page is live and in use: Games and screen-protection switches saved on 2026-10-13 (audit app_release.changed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Games (Admin and above)</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>Improvement</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H19" s="11" t="inlineStr">
+        <is>
+          <t>Games page: the limits the server enforces (largest bet, daily loss and win, payout multiple, launch lifetime, minimum age), the games received from Tulasi with 'In the app' and 'In Tulasi' status, Hide or Show per game and Show all / Hide all (a Sync never undoes a hide), 14-day totals, two watch reports (winners who then gift, hosts receiving from winners) and every balance call.</t>
+        </is>
+      </c>
+      <c r="I19" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J19" s="11" t="n"/>
+      <c r="K19" s="11" t="inlineStr">
+        <is>
+          <t>Super Admin, Master</t>
+        </is>
+      </c>
+      <c r="L19" s="11" t="n"/>
+      <c r="M19" s="11" t="n"/>
+      <c r="N19" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="O19" s="11" t="n"/>
+      <c r="P19" s="11" t="inlineStr">
+        <is>
+          <t>panel main b37c27e; migrations 20261013100000 to 20261013140000</t>
+        </is>
+      </c>
+      <c r="Q19" s="11" t="inlineStr">
+        <is>
+          <t>Panel deploy, Database migration</t>
+        </is>
+      </c>
+      <c r="R19" s="11" t="inlineStr">
+        <is>
+          <t>Owner changed the Games switch from the panel 2026-10-13; the Hide / Show buttons were not yet used on production (Claude applied the same change by SQL)</t>
+        </is>
+      </c>
+      <c r="S19" s="11" t="inlineStr">
+        <is>
+          <t>Limits: left at the defaults by the owner's decision on 2026-10-14.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Application Config &gt; Release controls</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>Improvement</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>Release switches 'Games' and 'Block screenshots and screen recording' (feature flags the apps read; both default off).</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="n"/>
+      <c r="K20" s="11" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="L20" s="11" t="n"/>
+      <c r="M20" s="11" t="n"/>
+      <c r="N20" s="11" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="O20" s="11" t="n"/>
+      <c r="P20" s="11" t="inlineStr">
+        <is>
+          <t>panel part 1 (5e15bf4) and part 2 (b37c27e)</t>
+        </is>
+      </c>
+      <c r="Q20" s="11" t="inlineStr">
+        <is>
+          <t>Panel deploy</t>
+        </is>
+      </c>
+      <c r="R20" s="11" t="inlineStr">
+        <is>
+          <t>Owner 2026-10-13 (audit log app_release.changed at 13:30:24 on, 13:54:47 off, 14:01:10 on) and Claude (23 players launched games after the switch)</t>
+        </is>
+      </c>
+      <c r="S20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Content / Emotes &amp; GIFs, Application Config, landing site</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>Improvement</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H21" s="11" t="inlineStr">
+        <is>
+          <t>Panel release part 1: the Emoji pages are now Emotes &amp; GIFs, a live branding preview in Application Config, and the landing site reads its project from the environment (production by default).</t>
+        </is>
+      </c>
+      <c r="I21" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J21" s="11" t="n"/>
+      <c r="K21" s="11" t="inlineStr">
+        <is>
+          <t>Super Admin, Master</t>
+        </is>
+      </c>
+      <c r="L21" s="11" t="n"/>
+      <c r="M21" s="11" t="n"/>
+      <c r="N21" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="O21" s="11" t="n"/>
+      <c r="P21" s="11" t="inlineStr">
+        <is>
+          <t>panel main 5e15bf4 (2026-10-13)</t>
+        </is>
+      </c>
+      <c r="Q21" s="11" t="inlineStr">
+        <is>
+          <t>Panel deploy</t>
+        </is>
+      </c>
+      <c r="R21" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S21" s="11" t="inlineStr">
+        <is>
+          <t>Checked on the live bundle: new text present, none of the part-2 names.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>Store / Coins / Lucky Box</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>Improvement</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H22" s="11" t="inlineStr">
+        <is>
+          <t>Panel release part 2: effect play speed and sound fields on entry effects, vehicles and gifts; Lucky Box cooldown (hours) field.</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J22" s="11" t="n"/>
+      <c r="K22" s="11" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="L22" s="11" t="n"/>
+      <c r="M22" s="11" t="n"/>
+      <c r="N22" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="O22" s="11" t="n"/>
+      <c r="P22" s="11" t="inlineStr">
+        <is>
+          <t>panel main b37c27e; migrations 20261009120000, 20261010090000</t>
+        </is>
+      </c>
+      <c r="Q22" s="11" t="inlineStr">
+        <is>
+          <t>Panel deploy, Database migration</t>
+        </is>
+      </c>
+      <c r="R22" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S22" s="11" t="inlineStr">
+        <is>
+          <t>Applied on production 2026-10-13.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>View user profile &gt; assign / remove</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H23" s="11" t="inlineStr">
+        <is>
+          <t>The panel code for assign and remove on View user profile reached production on 2026-10-12, but its migration 20261012100000 did not, so removing a badge or frame would fail with 'function not found'. FIX: the migration was applied on 2026-10-13 07:19 UTC.</t>
+        </is>
+      </c>
+      <c r="I23" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J23" s="11" t="n"/>
+      <c r="K23" s="11" t="inlineStr">
+        <is>
+          <t>Super Admin, Master</t>
+        </is>
+      </c>
+      <c r="L23" s="11" t="n"/>
+      <c r="M23" s="11" t="n"/>
+      <c r="N23" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="O23" s="11" t="n"/>
+      <c r="P23" s="11" t="inlineStr">
+        <is>
+          <t>migration 20261012100000</t>
+        </is>
+      </c>
+      <c r="Q23" s="11" t="inlineStr">
+        <is>
+          <t>Database migration</t>
+        </is>
+      </c>
+      <c r="R23" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S23" s="11" t="inlineStr">
+        <is>
+          <t>Found by Claude during the part-1 release check; staff-only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Top bar</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>Improvement</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t>Master and Super Admin can switch the panel between the production and staging projects (each keeps its own session; staging shows an orange strip).</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="n"/>
+      <c r="K24" s="11" t="inlineStr">
+        <is>
+          <t>Super Admin, Master</t>
+        </is>
+      </c>
+      <c r="L24" s="11" t="n"/>
+      <c r="M24" s="11" t="n"/>
+      <c r="N24" s="11" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="O24" s="11" t="n"/>
+      <c r="P24" s="11" t="inlineStr">
+        <is>
+          <t>panel main 2778960 (2026-10-11)</t>
+        </is>
+      </c>
+      <c r="Q24" s="11" t="inlineStr">
+        <is>
+          <t>Panel deploy</t>
+        </is>
+      </c>
+      <c r="R24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S24" s="11" t="inlineStr">
+        <is>
+          <t>Needs the two staging variables in Vercel (set).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S18"/>
+  <autoFilter ref="A1:S24"/>
   <conditionalFormatting sqref="G2:G400">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Critical"</formula>

</xml_diff>